<commit_message>
Add --download-media: WebP photos <100KB and videos per product code
</commit_message>
<xml_diff>
--- a/Product Database - filled.xlsx
+++ b/Product Database - filled.xlsx
@@ -580,7 +580,11 @@
           <t>FA-1959</t>
         </is>
       </c>
-      <c r="C2" s="9" t="n"/>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>FA-1959-1.webp | FA-1959-2.webp | FA-1959-3.webp | FA-1959-4.webp | FA-1959-5.webp | FA-1959-6.webp | FA-1959-7.webp</t>
+        </is>
+      </c>
       <c r="D2" s="10" t="n"/>
       <c r="E2" s="20" t="inlineStr">
         <is>
@@ -646,7 +650,11 @@
           <t>FA-2209</t>
         </is>
       </c>
-      <c r="C3" s="9" t="n"/>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>FA-2209-1.webp | FA-2209-2.webp | FA-2209-3.webp | FA-2209-4.webp</t>
+        </is>
+      </c>
       <c r="D3" s="10" t="n"/>
       <c r="E3" s="20" t="inlineStr">
         <is>
@@ -708,7 +716,11 @@
           <t>FA-1990</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n"/>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>FA-1990-1.webp | FA-1990-2.webp | FA-1990-3.webp | FA-1990-4.webp | FA-1990-5.webp | FA-1990-6.webp</t>
+        </is>
+      </c>
       <c r="D4" s="10" t="n"/>
       <c r="E4" s="20" t="inlineStr">
         <is>
@@ -766,7 +778,11 @@
           <t>FA-1863</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n"/>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>FA-1863-1.webp | FA-1863-2.webp | FA-1863-3.webp | FA-1863-4.webp | FA-1863-5.webp | FA-1863-6.webp</t>
+        </is>
+      </c>
       <c r="D5" s="10" t="n"/>
       <c r="E5" s="20" t="inlineStr">
         <is>
@@ -882,7 +898,11 @@
           <t>FA-1868</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n"/>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>FA-1868-1.webp | FA-1868-2.webp | FA-1868-3.webp | FA-1868-4.webp | FA-1868-5.webp</t>
+        </is>
+      </c>
       <c r="D7" s="10" t="n"/>
       <c r="E7" s="20" t="inlineStr">
         <is>
@@ -998,7 +1018,11 @@
           <t>FA-1944</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n"/>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>FA-1944-1.webp | FA-1944-2.webp</t>
+        </is>
+      </c>
       <c r="D9" s="10" t="n"/>
       <c r="E9" s="20" t="inlineStr">
         <is>
@@ -1056,7 +1080,11 @@
           <t>FA-2024</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n"/>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>FA-2024-1.webp | FA-2024-2.webp | FA-2024-3.webp | FA-2024-4.webp | FA-2024-5.webp | FA-2024-6.webp | FA-2024-7.webp</t>
+        </is>
+      </c>
       <c r="D10" s="10" t="n"/>
       <c r="E10" s="20" t="n"/>
       <c r="F10" s="20" t="n"/>
@@ -1110,7 +1138,11 @@
           <t>FA-2093</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n"/>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>FA-2093-1.webp | FA-2093-2.webp | FA-2093-3.webp | FA-2093-4.webp | FA-2093-5.webp | FA-2093-6.webp | FA-2093-7.webp</t>
+        </is>
+      </c>
       <c r="D11" s="10" t="n"/>
       <c r="E11" s="20" t="n"/>
       <c r="F11" s="20" t="inlineStr">
@@ -1168,7 +1200,11 @@
           <t>FA-2091</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n"/>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>FA-2091-1.webp | FA-2091-2.webp | FA-2091-3.webp | FA-2091-4.webp | FA-2091-5.webp | FA-2091-6.webp | FA-2091-7.webp</t>
+        </is>
+      </c>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="20" t="inlineStr">
         <is>
@@ -1234,7 +1270,11 @@
           <t>SHK-649</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n"/>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>SHK-649-1.webp | SHK-649-2.webp | SHK-649-3.webp | SHK-649-4.webp | SHK-649-5.webp | SHK-649-6.webp</t>
+        </is>
+      </c>
       <c r="D13" s="10" t="n"/>
       <c r="E13" s="20" t="n"/>
       <c r="F13" s="20" t="inlineStr">
@@ -1308,7 +1348,11 @@
           <t>SHK-655</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n"/>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>SHK-655-1.webp | SHK-655-2.webp | SHK-655-3.webp</t>
+        </is>
+      </c>
       <c r="D14" s="10" t="n"/>
       <c r="E14" s="20" t="n"/>
       <c r="F14" s="20" t="inlineStr">
@@ -1382,7 +1426,11 @@
           <t>SHK-659</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n"/>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>SHK-659-1.webp | SHK-659-2.webp | SHK-659-3.webp | SHK-659-4.webp</t>
+        </is>
+      </c>
       <c r="D15" s="10" t="n"/>
       <c r="E15" s="20" t="n"/>
       <c r="F15" s="20" t="inlineStr">
@@ -1456,7 +1504,11 @@
           <t>SHK-680</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n"/>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>SHK-680-1.webp | SHK-680-2.webp | SHK-680-3.webp</t>
+        </is>
+      </c>
       <c r="D16" s="10" t="n"/>
       <c r="E16" s="20" t="n"/>
       <c r="F16" s="20" t="inlineStr">
@@ -1530,7 +1582,11 @@
           <t>BA-1482</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n"/>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>BA-1482-1.webp</t>
+        </is>
+      </c>
       <c r="D17" s="10" t="n"/>
       <c r="E17" s="20" t="inlineStr">
         <is>
@@ -1600,7 +1656,11 @@
           <t>BA-1981</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n"/>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>BA-1981-1.webp</t>
+        </is>
+      </c>
       <c r="D18" s="10" t="n"/>
       <c r="E18" s="20" t="inlineStr">
         <is>
@@ -1732,7 +1792,11 @@
           <t>BA-1488</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n"/>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>BA-1488-1.webp</t>
+        </is>
+      </c>
       <c r="D20" s="10" t="n"/>
       <c r="E20" s="20" t="inlineStr">
         <is>
@@ -1802,7 +1866,11 @@
           <t>BA-1486</t>
         </is>
       </c>
-      <c r="C21" s="20" t="n"/>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>BA-1486-1.webp</t>
+        </is>
+      </c>
       <c r="D21" s="10" t="n"/>
       <c r="E21" s="20" t="inlineStr">
         <is>
@@ -1872,7 +1940,11 @@
           <t>BA-1413</t>
         </is>
       </c>
-      <c r="C22" s="20" t="n"/>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>BA-1413-1.webp</t>
+        </is>
+      </c>
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="20" t="inlineStr">
         <is>
@@ -1946,7 +2018,11 @@
           <t>BA-1933</t>
         </is>
       </c>
-      <c r="C23" s="20" t="n"/>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>BA-1933-1.webp</t>
+        </is>
+      </c>
       <c r="D23" s="10" t="n"/>
       <c r="E23" s="20" t="inlineStr">
         <is>
@@ -2090,7 +2166,11 @@
           <t>BA-1494</t>
         </is>
       </c>
-      <c r="C25" s="20" t="n"/>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>BA-1494-1.webp</t>
+        </is>
+      </c>
       <c r="D25" s="10" t="n"/>
       <c r="E25" s="20" t="inlineStr">
         <is>
@@ -2160,7 +2240,11 @@
           <t>BA-1330</t>
         </is>
       </c>
-      <c r="C26" s="20" t="n"/>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>BA-1330-1.webp</t>
+        </is>
+      </c>
       <c r="D26" s="10" t="n"/>
       <c r="E26" s="20" t="inlineStr">
         <is>
@@ -2234,7 +2318,11 @@
           <t>BA-1280</t>
         </is>
       </c>
-      <c r="C27" s="20" t="n"/>
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>BA-1280-1.webp</t>
+        </is>
+      </c>
       <c r="D27" s="10" t="n"/>
       <c r="E27" s="20" t="inlineStr">
         <is>
@@ -2304,7 +2392,11 @@
           <t>BA-1442</t>
         </is>
       </c>
-      <c r="C28" s="20" t="n"/>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>BA-1442-1.webp</t>
+        </is>
+      </c>
       <c r="D28" s="10" t="n"/>
       <c r="E28" s="20" t="inlineStr">
         <is>
@@ -2490,7 +2582,11 @@
           <t>TR-402</t>
         </is>
       </c>
-      <c r="C31" s="20" t="n"/>
+      <c r="C31" s="20" t="inlineStr">
+        <is>
+          <t>TR-402-1.webp | TR-402-2.webp | TR-402-3.webp | TR-402-4.webp | TR-402-5.webp | TR-402-6.webp</t>
+        </is>
+      </c>
       <c r="D31" s="10" t="n"/>
       <c r="E31" s="20" t="inlineStr">
         <is>
@@ -2556,7 +2652,11 @@
           <t>TR-439</t>
         </is>
       </c>
-      <c r="C32" s="20" t="n"/>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>TR-439-1.webp | TR-439-2.webp | TR-439-3.webp | TR-439-4.webp</t>
+        </is>
+      </c>
       <c r="D32" s="10" t="n"/>
       <c r="E32" s="20" t="inlineStr">
         <is>
@@ -2622,7 +2722,11 @@
           <t>TR-429</t>
         </is>
       </c>
-      <c r="C33" s="20" t="n"/>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>TR-429-1.webp | TR-429-2.webp | TR-429-3.webp | TR-429-4.webp | TR-429-5.webp</t>
+        </is>
+      </c>
       <c r="D33" s="10" t="n"/>
       <c r="E33" s="20" t="inlineStr">
         <is>
@@ -2688,7 +2792,11 @@
           <t>TR-258</t>
         </is>
       </c>
-      <c r="C34" s="20" t="n"/>
+      <c r="C34" s="20" t="inlineStr">
+        <is>
+          <t>TR-258-1.webp | TR-258-2.webp | TR-258-3.webp | TR-258-4.webp | TR-258-5.webp</t>
+        </is>
+      </c>
       <c r="D34" s="10" t="n"/>
       <c r="E34" s="20" t="inlineStr">
         <is>
@@ -2812,7 +2920,11 @@
           <t>TR-445</t>
         </is>
       </c>
-      <c r="C36" s="20" t="n"/>
+      <c r="C36" s="20" t="inlineStr">
+        <is>
+          <t>TR-445-1.webp | TR-445-2.webp | TR-445-3.webp | TR-445-4.webp | TR-445-5.webp | TR-445-6.webp</t>
+        </is>
+      </c>
       <c r="D36" s="10" t="n"/>
       <c r="E36" s="20" t="inlineStr">
         <is>
@@ -2878,7 +2990,11 @@
           <t>TR-358</t>
         </is>
       </c>
-      <c r="C37" s="20" t="n"/>
+      <c r="C37" s="20" t="inlineStr">
+        <is>
+          <t>TR-358-1.webp | TR-358-2.webp | TR-358-3.webp | TR-358-4.webp | TR-358-5.webp | TR-358-6.webp | TR-358-7.webp</t>
+        </is>
+      </c>
       <c r="D37" s="10" t="n"/>
       <c r="E37" s="20" t="inlineStr">
         <is>
@@ -2998,7 +3114,11 @@
           <t>MR-5014</t>
         </is>
       </c>
-      <c r="C39" s="20" t="n"/>
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t>MR-5014-1.webp | MR-5014-2.webp | MR-5014-3.webp | MR-5014-4.webp | MR-5014-5.webp | MR-5014-6.webp</t>
+        </is>
+      </c>
       <c r="D39" s="10" t="n"/>
       <c r="E39" s="20" t="n"/>
       <c r="F39" s="20" t="n"/>
@@ -3114,7 +3234,11 @@
           <t>MR-5167</t>
         </is>
       </c>
-      <c r="C41" s="20" t="n"/>
+      <c r="C41" s="20" t="inlineStr">
+        <is>
+          <t>MR-5167-1.webp | MR-5167-2.webp | MR-5167-3.webp | MR-5167-4.webp</t>
+        </is>
+      </c>
       <c r="D41" s="10" t="n"/>
       <c r="E41" s="20" t="n"/>
       <c r="F41" s="20" t="n"/>
@@ -3176,7 +3300,11 @@
           <t>MR-5083</t>
         </is>
       </c>
-      <c r="C42" s="20" t="n"/>
+      <c r="C42" s="20" t="inlineStr">
+        <is>
+          <t>MR-5083-1.webp | MR-5083-2.webp | MR-5083-3.webp | MR-5083-4.webp | MR-5083-5.webp | MR-5083-6.webp | MR-5083-7.webp</t>
+        </is>
+      </c>
       <c r="D42" s="10" t="n"/>
       <c r="E42" s="20" t="n"/>
       <c r="F42" s="20" t="n"/>

</xml_diff>

<commit_message>
Incremental reruns: media manifest, --refresh, graceful offline failure
</commit_message>
<xml_diff>
--- a/Product Database - filled.xlsx
+++ b/Product Database - filled.xlsx
@@ -580,11 +580,7 @@
           <t>FA-1959</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>FA-1959-1.webp | FA-1959-2.webp | FA-1959-3.webp | FA-1959-4.webp | FA-1959-5.webp | FA-1959-6.webp | FA-1959-7.webp</t>
-        </is>
-      </c>
+      <c r="C2" s="9" t="n"/>
       <c r="D2" s="10" t="n"/>
       <c r="E2" s="20" t="inlineStr">
         <is>
@@ -650,11 +646,7 @@
           <t>FA-2209</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>FA-2209-1.webp | FA-2209-2.webp | FA-2209-3.webp | FA-2209-4.webp</t>
-        </is>
-      </c>
+      <c r="C3" s="9" t="n"/>
       <c r="D3" s="10" t="n"/>
       <c r="E3" s="20" t="inlineStr">
         <is>
@@ -716,11 +708,7 @@
           <t>FA-1990</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>FA-1990-1.webp | FA-1990-2.webp | FA-1990-3.webp | FA-1990-4.webp | FA-1990-5.webp | FA-1990-6.webp</t>
-        </is>
-      </c>
+      <c r="C4" s="9" t="n"/>
       <c r="D4" s="10" t="n"/>
       <c r="E4" s="20" t="inlineStr">
         <is>
@@ -778,11 +766,7 @@
           <t>FA-1863</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
-        <is>
-          <t>FA-1863-1.webp | FA-1863-2.webp | FA-1863-3.webp | FA-1863-4.webp | FA-1863-5.webp | FA-1863-6.webp</t>
-        </is>
-      </c>
+      <c r="C5" s="20" t="n"/>
       <c r="D5" s="10" t="n"/>
       <c r="E5" s="20" t="inlineStr">
         <is>
@@ -898,11 +882,7 @@
           <t>FA-1868</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>FA-1868-1.webp | FA-1868-2.webp | FA-1868-3.webp | FA-1868-4.webp | FA-1868-5.webp</t>
-        </is>
-      </c>
+      <c r="C7" s="20" t="n"/>
       <c r="D7" s="10" t="n"/>
       <c r="E7" s="20" t="inlineStr">
         <is>
@@ -1018,11 +998,7 @@
           <t>FA-1944</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
-        <is>
-          <t>FA-1944-1.webp | FA-1944-2.webp</t>
-        </is>
-      </c>
+      <c r="C9" s="20" t="n"/>
       <c r="D9" s="10" t="n"/>
       <c r="E9" s="20" t="inlineStr">
         <is>
@@ -1080,11 +1056,7 @@
           <t>FA-2024</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>FA-2024-1.webp | FA-2024-2.webp | FA-2024-3.webp | FA-2024-4.webp | FA-2024-5.webp | FA-2024-6.webp | FA-2024-7.webp</t>
-        </is>
-      </c>
+      <c r="C10" s="20" t="n"/>
       <c r="D10" s="10" t="n"/>
       <c r="E10" s="20" t="n"/>
       <c r="F10" s="20" t="n"/>
@@ -1138,11 +1110,7 @@
           <t>FA-2093</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>FA-2093-1.webp | FA-2093-2.webp | FA-2093-3.webp | FA-2093-4.webp | FA-2093-5.webp | FA-2093-6.webp | FA-2093-7.webp</t>
-        </is>
-      </c>
+      <c r="C11" s="20" t="n"/>
       <c r="D11" s="10" t="n"/>
       <c r="E11" s="20" t="n"/>
       <c r="F11" s="20" t="inlineStr">
@@ -1200,11 +1168,7 @@
           <t>FA-2091</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>FA-2091-1.webp | FA-2091-2.webp | FA-2091-3.webp | FA-2091-4.webp | FA-2091-5.webp | FA-2091-6.webp | FA-2091-7.webp</t>
-        </is>
-      </c>
+      <c r="C12" s="20" t="n"/>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="20" t="inlineStr">
         <is>
@@ -1270,11 +1234,7 @@
           <t>SHK-649</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
-        <is>
-          <t>SHK-649-1.webp | SHK-649-2.webp | SHK-649-3.webp | SHK-649-4.webp | SHK-649-5.webp | SHK-649-6.webp</t>
-        </is>
-      </c>
+      <c r="C13" s="20" t="n"/>
       <c r="D13" s="10" t="n"/>
       <c r="E13" s="20" t="n"/>
       <c r="F13" s="20" t="inlineStr">
@@ -1348,11 +1308,7 @@
           <t>SHK-655</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
-        <is>
-          <t>SHK-655-1.webp | SHK-655-2.webp | SHK-655-3.webp</t>
-        </is>
-      </c>
+      <c r="C14" s="20" t="n"/>
       <c r="D14" s="10" t="n"/>
       <c r="E14" s="20" t="n"/>
       <c r="F14" s="20" t="inlineStr">
@@ -1426,11 +1382,7 @@
           <t>SHK-659</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>SHK-659-1.webp | SHK-659-2.webp | SHK-659-3.webp | SHK-659-4.webp</t>
-        </is>
-      </c>
+      <c r="C15" s="20" t="n"/>
       <c r="D15" s="10" t="n"/>
       <c r="E15" s="20" t="n"/>
       <c r="F15" s="20" t="inlineStr">
@@ -1504,11 +1456,7 @@
           <t>SHK-680</t>
         </is>
       </c>
-      <c r="C16" s="20" t="inlineStr">
-        <is>
-          <t>SHK-680-1.webp | SHK-680-2.webp | SHK-680-3.webp</t>
-        </is>
-      </c>
+      <c r="C16" s="20" t="n"/>
       <c r="D16" s="10" t="n"/>
       <c r="E16" s="20" t="n"/>
       <c r="F16" s="20" t="inlineStr">
@@ -1582,11 +1530,7 @@
           <t>BA-1482</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
-        <is>
-          <t>BA-1482-1.webp</t>
-        </is>
-      </c>
+      <c r="C17" s="20" t="n"/>
       <c r="D17" s="10" t="n"/>
       <c r="E17" s="20" t="inlineStr">
         <is>
@@ -1656,11 +1600,7 @@
           <t>BA-1981</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
-        <is>
-          <t>BA-1981-1.webp</t>
-        </is>
-      </c>
+      <c r="C18" s="20" t="n"/>
       <c r="D18" s="10" t="n"/>
       <c r="E18" s="20" t="inlineStr">
         <is>
@@ -1792,11 +1732,7 @@
           <t>BA-1488</t>
         </is>
       </c>
-      <c r="C20" s="20" t="inlineStr">
-        <is>
-          <t>BA-1488-1.webp</t>
-        </is>
-      </c>
+      <c r="C20" s="20" t="n"/>
       <c r="D20" s="10" t="n"/>
       <c r="E20" s="20" t="inlineStr">
         <is>
@@ -1866,11 +1802,7 @@
           <t>BA-1486</t>
         </is>
       </c>
-      <c r="C21" s="20" t="inlineStr">
-        <is>
-          <t>BA-1486-1.webp</t>
-        </is>
-      </c>
+      <c r="C21" s="20" t="n"/>
       <c r="D21" s="10" t="n"/>
       <c r="E21" s="20" t="inlineStr">
         <is>
@@ -1940,11 +1872,7 @@
           <t>BA-1413</t>
         </is>
       </c>
-      <c r="C22" s="20" t="inlineStr">
-        <is>
-          <t>BA-1413-1.webp</t>
-        </is>
-      </c>
+      <c r="C22" s="20" t="n"/>
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="20" t="inlineStr">
         <is>
@@ -2018,11 +1946,7 @@
           <t>BA-1933</t>
         </is>
       </c>
-      <c r="C23" s="20" t="inlineStr">
-        <is>
-          <t>BA-1933-1.webp</t>
-        </is>
-      </c>
+      <c r="C23" s="20" t="n"/>
       <c r="D23" s="10" t="n"/>
       <c r="E23" s="20" t="inlineStr">
         <is>
@@ -2166,11 +2090,7 @@
           <t>BA-1494</t>
         </is>
       </c>
-      <c r="C25" s="20" t="inlineStr">
-        <is>
-          <t>BA-1494-1.webp</t>
-        </is>
-      </c>
+      <c r="C25" s="20" t="n"/>
       <c r="D25" s="10" t="n"/>
       <c r="E25" s="20" t="inlineStr">
         <is>
@@ -2240,11 +2160,7 @@
           <t>BA-1330</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
-        <is>
-          <t>BA-1330-1.webp</t>
-        </is>
-      </c>
+      <c r="C26" s="20" t="n"/>
       <c r="D26" s="10" t="n"/>
       <c r="E26" s="20" t="inlineStr">
         <is>
@@ -2318,11 +2234,7 @@
           <t>BA-1280</t>
         </is>
       </c>
-      <c r="C27" s="20" t="inlineStr">
-        <is>
-          <t>BA-1280-1.webp</t>
-        </is>
-      </c>
+      <c r="C27" s="20" t="n"/>
       <c r="D27" s="10" t="n"/>
       <c r="E27" s="20" t="inlineStr">
         <is>
@@ -2392,11 +2304,7 @@
           <t>BA-1442</t>
         </is>
       </c>
-      <c r="C28" s="20" t="inlineStr">
-        <is>
-          <t>BA-1442-1.webp</t>
-        </is>
-      </c>
+      <c r="C28" s="20" t="n"/>
       <c r="D28" s="10" t="n"/>
       <c r="E28" s="20" t="inlineStr">
         <is>
@@ -2582,11 +2490,7 @@
           <t>TR-402</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
-        <is>
-          <t>TR-402-1.webp | TR-402-2.webp | TR-402-3.webp | TR-402-4.webp | TR-402-5.webp | TR-402-6.webp</t>
-        </is>
-      </c>
+      <c r="C31" s="20" t="n"/>
       <c r="D31" s="10" t="n"/>
       <c r="E31" s="20" t="inlineStr">
         <is>
@@ -2652,11 +2556,7 @@
           <t>TR-439</t>
         </is>
       </c>
-      <c r="C32" s="20" t="inlineStr">
-        <is>
-          <t>TR-439-1.webp | TR-439-2.webp | TR-439-3.webp | TR-439-4.webp</t>
-        </is>
-      </c>
+      <c r="C32" s="20" t="n"/>
       <c r="D32" s="10" t="n"/>
       <c r="E32" s="20" t="inlineStr">
         <is>
@@ -2722,11 +2622,7 @@
           <t>TR-429</t>
         </is>
       </c>
-      <c r="C33" s="20" t="inlineStr">
-        <is>
-          <t>TR-429-1.webp | TR-429-2.webp | TR-429-3.webp | TR-429-4.webp | TR-429-5.webp</t>
-        </is>
-      </c>
+      <c r="C33" s="20" t="n"/>
       <c r="D33" s="10" t="n"/>
       <c r="E33" s="20" t="inlineStr">
         <is>
@@ -2792,11 +2688,7 @@
           <t>TR-258</t>
         </is>
       </c>
-      <c r="C34" s="20" t="inlineStr">
-        <is>
-          <t>TR-258-1.webp | TR-258-2.webp | TR-258-3.webp | TR-258-4.webp | TR-258-5.webp</t>
-        </is>
-      </c>
+      <c r="C34" s="20" t="n"/>
       <c r="D34" s="10" t="n"/>
       <c r="E34" s="20" t="inlineStr">
         <is>
@@ -2920,11 +2812,7 @@
           <t>TR-445</t>
         </is>
       </c>
-      <c r="C36" s="20" t="inlineStr">
-        <is>
-          <t>TR-445-1.webp | TR-445-2.webp | TR-445-3.webp | TR-445-4.webp | TR-445-5.webp | TR-445-6.webp</t>
-        </is>
-      </c>
+      <c r="C36" s="20" t="n"/>
       <c r="D36" s="10" t="n"/>
       <c r="E36" s="20" t="inlineStr">
         <is>
@@ -2990,11 +2878,7 @@
           <t>TR-358</t>
         </is>
       </c>
-      <c r="C37" s="20" t="inlineStr">
-        <is>
-          <t>TR-358-1.webp | TR-358-2.webp | TR-358-3.webp | TR-358-4.webp | TR-358-5.webp | TR-358-6.webp | TR-358-7.webp</t>
-        </is>
-      </c>
+      <c r="C37" s="20" t="n"/>
       <c r="D37" s="10" t="n"/>
       <c r="E37" s="20" t="inlineStr">
         <is>
@@ -3114,11 +2998,7 @@
           <t>MR-5014</t>
         </is>
       </c>
-      <c r="C39" s="20" t="inlineStr">
-        <is>
-          <t>MR-5014-1.webp | MR-5014-2.webp | MR-5014-3.webp | MR-5014-4.webp | MR-5014-5.webp | MR-5014-6.webp</t>
-        </is>
-      </c>
+      <c r="C39" s="20" t="n"/>
       <c r="D39" s="10" t="n"/>
       <c r="E39" s="20" t="n"/>
       <c r="F39" s="20" t="n"/>
@@ -3234,11 +3114,7 @@
           <t>MR-5167</t>
         </is>
       </c>
-      <c r="C41" s="20" t="inlineStr">
-        <is>
-          <t>MR-5167-1.webp | MR-5167-2.webp | MR-5167-3.webp | MR-5167-4.webp</t>
-        </is>
-      </c>
+      <c r="C41" s="20" t="n"/>
       <c r="D41" s="10" t="n"/>
       <c r="E41" s="20" t="n"/>
       <c r="F41" s="20" t="n"/>
@@ -3300,11 +3176,7 @@
           <t>MR-5083</t>
         </is>
       </c>
-      <c r="C42" s="20" t="inlineStr">
-        <is>
-          <t>MR-5083-1.webp | MR-5083-2.webp | MR-5083-3.webp | MR-5083-4.webp | MR-5083-5.webp | MR-5083-6.webp | MR-5083-7.webp</t>
-        </is>
-      </c>
+      <c r="C42" s="20" t="n"/>
       <c r="D42" s="10" t="n"/>
       <c r="E42" s="20" t="n"/>
       <c r="F42" s="20" t="n"/>

</xml_diff>